<commit_message>
MAJ v5.1 : référence gabarits vs LLM ancré, résumé avec moteur et modèle, documentation
- évaluation : commentaires en mode gabarits et LLM ancré comparés aux commentaires publiés
  (ROUGE-L, similarité, couverture, Wilcoxon) ; côté gabarits mesuré, côté LLM non mesuré ici
- grille BN : notes stratégiques des deux versions ; figure gabarits vs LLM
- resume.md et manifest : moteur et modèle explicites ; Tableau 3.2 : 4 candidats Ollama + Groq
- docs : nouveau titre, double moteur, installation Groq (développement), écarts E11-E14, valeurs mises à jour
- test : le moteur livré est local

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013JXMEQCNGgRjDzvz3X6fC9
</commit_message>
<xml_diff>
--- a/data/results/2026-09-28/h3_grille_evaluation.xlsx
+++ b/data/results/2026-09-28/h3_grille_evaluation.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -477,16 +477,21 @@
           <t>remarques</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>version</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Note d'analyse stratégique — exercice 2024</t>
+          <t>Note d'analyse stratégique — exercice 2024 — gabarits</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>note_strategique_2024.docx</t>
+          <t>note_strategique_2024_gabarits.docx</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -505,16 +510,21 @@
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>gabarits</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Note d'analyse stratégique — exercice 2024</t>
+          <t>Note d'analyse stratégique — exercice 2024 — gabarits</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>note_strategique_2024.docx</t>
+          <t>note_strategique_2024_gabarits.docx</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -533,16 +543,21 @@
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>gabarits</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Note d'analyse stratégique — exercice 2024</t>
+          <t>Note d'analyse stratégique — exercice 2024 — gabarits</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>note_strategique_2024.docx</t>
+          <t>note_strategique_2024_gabarits.docx</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -561,16 +576,21 @@
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>gabarits</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Note d'analyse stratégique — exercice 2024</t>
+          <t>Note d'analyse stratégique — exercice 2024 — gabarits</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>note_strategique_2024.docx</t>
+          <t>note_strategique_2024_gabarits.docx</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -589,16 +609,21 @@
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>gabarits</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Note d'analyse stratégique — exercice 2024</t>
+          <t>Note d'analyse stratégique — exercice 2024 — gabarits</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>note_strategique_2024.docx</t>
+          <t>note_strategique_2024_gabarits.docx</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -617,16 +642,21 @@
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>gabarits</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Note d'analyse stratégique — exercice 2023</t>
+          <t>Note d'analyse stratégique — exercice 2023 — gabarits</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>note_strategique_2023.docx</t>
+          <t>note_strategique_2023_gabarits.docx</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -645,16 +675,21 @@
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>gabarits</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Note d'analyse stratégique — exercice 2023</t>
+          <t>Note d'analyse stratégique — exercice 2023 — gabarits</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>note_strategique_2023.docx</t>
+          <t>note_strategique_2023_gabarits.docx</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -673,16 +708,21 @@
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>gabarits</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Note d'analyse stratégique — exercice 2023</t>
+          <t>Note d'analyse stratégique — exercice 2023 — gabarits</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>note_strategique_2023.docx</t>
+          <t>note_strategique_2023_gabarits.docx</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -701,16 +741,21 @@
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>gabarits</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Note d'analyse stratégique — exercice 2023</t>
+          <t>Note d'analyse stratégique — exercice 2023 — gabarits</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>note_strategique_2023.docx</t>
+          <t>note_strategique_2023_gabarits.docx</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -729,16 +774,21 @@
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>gabarits</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Note d'analyse stratégique — exercice 2023</t>
+          <t>Note d'analyse stratégique — exercice 2023 — gabarits</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>note_strategique_2023.docx</t>
+          <t>note_strategique_2023_gabarits.docx</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -757,6 +807,11 @@
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>gabarits</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>